<commit_message>
Update: data for 20260429, regenerated reports
</commit_message>
<xml_diff>
--- a/f_total_cap_nhat.xlsx
+++ b/f_total_cap_nhat.xlsx
@@ -535,13 +535,13 @@
         <v>150469</v>
       </c>
       <c r="L2" t="n">
-        <v>67491</v>
+        <v>77543</v>
       </c>
       <c r="M2" t="n">
-        <v>15230</v>
+        <v>18149</v>
       </c>
       <c r="N2" t="n">
-        <v>52261</v>
+        <v>59394</v>
       </c>
     </row>
     <row r="3">
@@ -579,13 +579,13 @@
         <v>81428</v>
       </c>
       <c r="L3" t="n">
-        <v>108267</v>
+        <v>124018</v>
       </c>
       <c r="M3" t="n">
-        <v>43897</v>
+        <v>51469</v>
       </c>
       <c r="N3" t="n">
-        <v>64370</v>
+        <v>72549</v>
       </c>
     </row>
     <row r="4">
@@ -623,13 +623,13 @@
         <v>18713</v>
       </c>
       <c r="L4" t="n">
-        <v>19849</v>
+        <v>22541</v>
       </c>
       <c r="M4" t="n">
-        <v>3583</v>
+        <v>4275</v>
       </c>
       <c r="N4" t="n">
-        <v>16266</v>
+        <v>18266</v>
       </c>
     </row>
     <row r="5">
@@ -667,13 +667,13 @@
         <v>42408</v>
       </c>
       <c r="L5" t="n">
-        <v>24840</v>
+        <v>28201</v>
       </c>
       <c r="M5" t="n">
-        <v>6742</v>
+        <v>7661</v>
       </c>
       <c r="N5" t="n">
-        <v>18098</v>
+        <v>20540</v>
       </c>
     </row>
     <row r="6">
@@ -711,13 +711,13 @@
         <v>117439</v>
       </c>
       <c r="L6" t="n">
-        <v>71428</v>
+        <v>81432</v>
       </c>
       <c r="M6" t="n">
-        <v>16777</v>
+        <v>19477</v>
       </c>
       <c r="N6" t="n">
-        <v>54651</v>
+        <v>61955</v>
       </c>
     </row>
     <row r="7">
@@ -755,13 +755,13 @@
         <v>19076</v>
       </c>
       <c r="L7" t="n">
-        <v>9944</v>
+        <v>11156</v>
       </c>
       <c r="M7" t="n">
-        <v>1649</v>
+        <v>1914</v>
       </c>
       <c r="N7" t="n">
-        <v>8295</v>
+        <v>9242</v>
       </c>
     </row>
     <row r="8">
@@ -799,13 +799,13 @@
         <v>83014</v>
       </c>
       <c r="L8" t="n">
-        <v>66979</v>
+        <v>76229</v>
       </c>
       <c r="M8" t="n">
-        <v>14900</v>
+        <v>17609</v>
       </c>
       <c r="N8" t="n">
-        <v>52079</v>
+        <v>58620</v>
       </c>
     </row>
     <row r="9">
@@ -843,13 +843,13 @@
         <v>65107</v>
       </c>
       <c r="L9" t="n">
-        <v>50146</v>
+        <v>57115</v>
       </c>
       <c r="M9" t="n">
-        <v>15378</v>
+        <v>18127</v>
       </c>
       <c r="N9" t="n">
-        <v>34768</v>
+        <v>38988</v>
       </c>
     </row>
     <row r="10">
@@ -887,13 +887,13 @@
         <v>151451</v>
       </c>
       <c r="L10" t="n">
-        <v>93311</v>
+        <v>105517</v>
       </c>
       <c r="M10" t="n">
-        <v>31174</v>
+        <v>35942</v>
       </c>
       <c r="N10" t="n">
-        <v>62137</v>
+        <v>69575</v>
       </c>
     </row>
     <row r="11">
@@ -931,13 +931,13 @@
         <v>127517</v>
       </c>
       <c r="L11" t="n">
-        <v>67238</v>
+        <v>77837</v>
       </c>
       <c r="M11" t="n">
-        <v>16442</v>
+        <v>19426</v>
       </c>
       <c r="N11" t="n">
-        <v>50796</v>
+        <v>58411</v>
       </c>
     </row>
     <row r="12">
@@ -975,13 +975,13 @@
         <v>122266</v>
       </c>
       <c r="L12" t="n">
-        <v>80754</v>
+        <v>90980</v>
       </c>
       <c r="M12" t="n">
-        <v>15507</v>
+        <v>18585</v>
       </c>
       <c r="N12" t="n">
-        <v>65247</v>
+        <v>72395</v>
       </c>
     </row>
     <row r="13">
@@ -1019,13 +1019,13 @@
         <v>399425</v>
       </c>
       <c r="L13" t="n">
-        <v>215088</v>
+        <v>251605</v>
       </c>
       <c r="M13" t="n">
-        <v>107015</v>
+        <v>123936</v>
       </c>
       <c r="N13" t="n">
-        <v>108073</v>
+        <v>127669</v>
       </c>
     </row>
     <row r="14">
@@ -1063,13 +1063,13 @@
         <v>274795</v>
       </c>
       <c r="L14" t="n">
-        <v>240276</v>
+        <v>284549</v>
       </c>
       <c r="M14" t="n">
-        <v>115973</v>
+        <v>137420</v>
       </c>
       <c r="N14" t="n">
-        <v>124303</v>
+        <v>147129</v>
       </c>
     </row>
     <row r="15">
@@ -1107,13 +1107,13 @@
         <v>80530</v>
       </c>
       <c r="L15" t="n">
-        <v>75718</v>
+        <v>86966</v>
       </c>
       <c r="M15" t="n">
-        <v>26878</v>
+        <v>31265</v>
       </c>
       <c r="N15" t="n">
-        <v>48840</v>
+        <v>55701</v>
       </c>
     </row>
     <row r="16">
@@ -1151,13 +1151,13 @@
         <v>15975</v>
       </c>
       <c r="L16" t="n">
-        <v>51316</v>
+        <v>56679</v>
       </c>
       <c r="M16" t="n">
-        <v>7910</v>
+        <v>9262</v>
       </c>
       <c r="N16" t="n">
-        <v>43406</v>
+        <v>47417</v>
       </c>
     </row>
     <row r="17">
@@ -1195,13 +1195,13 @@
         <v>26564</v>
       </c>
       <c r="L17" t="n">
-        <v>26726</v>
+        <v>30510</v>
       </c>
       <c r="M17" t="n">
-        <v>7541</v>
+        <v>8858</v>
       </c>
       <c r="N17" t="n">
-        <v>19185</v>
+        <v>21652</v>
       </c>
     </row>
     <row r="18">
@@ -1239,13 +1239,13 @@
         <v>66764</v>
       </c>
       <c r="L18" t="n">
-        <v>70870</v>
+        <v>81004</v>
       </c>
       <c r="M18" t="n">
-        <v>21736</v>
+        <v>25646</v>
       </c>
       <c r="N18" t="n">
-        <v>49134</v>
+        <v>55358</v>
       </c>
     </row>
     <row r="19">
@@ -1283,13 +1283,13 @@
         <v>55231</v>
       </c>
       <c r="L19" t="n">
-        <v>43592</v>
+        <v>49519</v>
       </c>
       <c r="M19" t="n">
-        <v>12626</v>
+        <v>14742</v>
       </c>
       <c r="N19" t="n">
-        <v>30966</v>
+        <v>34777</v>
       </c>
     </row>
     <row r="20">
@@ -1327,13 +1327,13 @@
         <v>58737</v>
       </c>
       <c r="L20" t="n">
-        <v>40208</v>
+        <v>47231</v>
       </c>
       <c r="M20" t="n">
-        <v>10492</v>
+        <v>12557</v>
       </c>
       <c r="N20" t="n">
-        <v>29716</v>
+        <v>34674</v>
       </c>
     </row>
     <row r="21">
@@ -1371,13 +1371,13 @@
         <v>24382</v>
       </c>
       <c r="L21" t="n">
-        <v>15632</v>
+        <v>18358</v>
       </c>
       <c r="M21" t="n">
-        <v>4284</v>
+        <v>5128</v>
       </c>
       <c r="N21" t="n">
-        <v>11348</v>
+        <v>13230</v>
       </c>
     </row>
     <row r="22">
@@ -1415,13 +1415,13 @@
         <v>152229</v>
       </c>
       <c r="L22" t="n">
-        <v>79087</v>
+        <v>91008</v>
       </c>
       <c r="M22" t="n">
-        <v>21671</v>
+        <v>25839</v>
       </c>
       <c r="N22" t="n">
-        <v>57416</v>
+        <v>65169</v>
       </c>
     </row>
     <row r="23">
@@ -1459,13 +1459,13 @@
         <v>40867</v>
       </c>
       <c r="L23" t="n">
-        <v>28778</v>
+        <v>33044</v>
       </c>
       <c r="M23" t="n">
-        <v>6804</v>
+        <v>8117</v>
       </c>
       <c r="N23" t="n">
-        <v>21974</v>
+        <v>24927</v>
       </c>
     </row>
     <row r="24">
@@ -1503,13 +1503,13 @@
         <v>88798</v>
       </c>
       <c r="L24" t="n">
-        <v>94007</v>
+        <v>106760</v>
       </c>
       <c r="M24" t="n">
-        <v>22133</v>
+        <v>26787</v>
       </c>
       <c r="N24" t="n">
-        <v>71874</v>
+        <v>79973</v>
       </c>
     </row>
     <row r="25">
@@ -1547,13 +1547,13 @@
         <v>86600</v>
       </c>
       <c r="L25" t="n">
-        <v>64398</v>
+        <v>74479</v>
       </c>
       <c r="M25" t="n">
-        <v>22189</v>
+        <v>26124</v>
       </c>
       <c r="N25" t="n">
-        <v>42209</v>
+        <v>48355</v>
       </c>
     </row>
     <row r="26">
@@ -1591,13 +1591,13 @@
         <v>95605</v>
       </c>
       <c r="L26" t="n">
-        <v>97934</v>
+        <v>114529</v>
       </c>
       <c r="M26" t="n">
-        <v>32443</v>
+        <v>39114</v>
       </c>
       <c r="N26" t="n">
-        <v>65491</v>
+        <v>75415</v>
       </c>
     </row>
     <row r="27">
@@ -1635,13 +1635,13 @@
         <v>35197</v>
       </c>
       <c r="L27" t="n">
-        <v>35008</v>
+        <v>40234</v>
       </c>
       <c r="M27" t="n">
-        <v>10112</v>
+        <v>11858</v>
       </c>
       <c r="N27" t="n">
-        <v>24896</v>
+        <v>28376</v>
       </c>
     </row>
     <row r="28">
@@ -1679,13 +1679,13 @@
         <v>52800</v>
       </c>
       <c r="L28" t="n">
-        <v>50053</v>
+        <v>56855</v>
       </c>
       <c r="M28" t="n">
-        <v>8481</v>
+        <v>10163</v>
       </c>
       <c r="N28" t="n">
-        <v>41572</v>
+        <v>46692</v>
       </c>
     </row>
     <row r="29">
@@ -1723,13 +1723,13 @@
         <v>34093</v>
       </c>
       <c r="L29" t="n">
-        <v>32058</v>
+        <v>36559</v>
       </c>
       <c r="M29" t="n">
-        <v>5450</v>
+        <v>6482</v>
       </c>
       <c r="N29" t="n">
-        <v>26608</v>
+        <v>30077</v>
       </c>
     </row>
     <row r="30">
@@ -1767,13 +1767,13 @@
         <v>59519</v>
       </c>
       <c r="L30" t="n">
-        <v>30744</v>
+        <v>35366</v>
       </c>
       <c r="M30" t="n">
-        <v>5934</v>
+        <v>7164</v>
       </c>
       <c r="N30" t="n">
-        <v>24810</v>
+        <v>28202</v>
       </c>
     </row>
     <row r="31">
@@ -1811,13 +1811,13 @@
         <v>111215</v>
       </c>
       <c r="L31" t="n">
-        <v>67843</v>
+        <v>77984</v>
       </c>
       <c r="M31" t="n">
-        <v>16543</v>
+        <v>19970</v>
       </c>
       <c r="N31" t="n">
-        <v>51300</v>
+        <v>58014</v>
       </c>
     </row>
     <row r="32">
@@ -1855,13 +1855,13 @@
         <v>135620</v>
       </c>
       <c r="L32" t="n">
-        <v>73512</v>
+        <v>84651</v>
       </c>
       <c r="M32" t="n">
-        <v>18187</v>
+        <v>20965</v>
       </c>
       <c r="N32" t="n">
-        <v>55325</v>
+        <v>63686</v>
       </c>
     </row>
     <row r="33">
@@ -1899,13 +1899,13 @@
         <v>46108</v>
       </c>
       <c r="L33" t="n">
-        <v>48923</v>
+        <v>56833</v>
       </c>
       <c r="M33" t="n">
-        <v>16731</v>
+        <v>19978</v>
       </c>
       <c r="N33" t="n">
-        <v>32192</v>
+        <v>36855</v>
       </c>
     </row>
     <row r="34">
@@ -1943,13 +1943,13 @@
         <v>74035</v>
       </c>
       <c r="L34" t="n">
-        <v>48207</v>
+        <v>56342</v>
       </c>
       <c r="M34" t="n">
-        <v>10666</v>
+        <v>12814</v>
       </c>
       <c r="N34" t="n">
-        <v>37541</v>
+        <v>43528</v>
       </c>
     </row>
     <row r="35">
@@ -1987,13 +1987,13 @@
         <v>134411</v>
       </c>
       <c r="L35" t="n">
-        <v>72687</v>
+        <v>84616</v>
       </c>
       <c r="M35" t="n">
-        <v>14782</v>
+        <v>17861</v>
       </c>
       <c r="N35" t="n">
-        <v>57905</v>
+        <v>66755</v>
       </c>
     </row>
     <row r="36">
@@ -2031,13 +2031,13 @@
         <v>93875</v>
       </c>
       <c r="L36" t="n">
-        <v>54068</v>
+        <v>61912</v>
       </c>
       <c r="M36" t="n">
-        <v>10539</v>
+        <v>12594</v>
       </c>
       <c r="N36" t="n">
-        <v>43529</v>
+        <v>49318</v>
       </c>
     </row>
     <row r="37">
@@ -2075,13 +2075,13 @@
         <v>65690</v>
       </c>
       <c r="L37" t="n">
-        <v>83403</v>
+        <v>95188</v>
       </c>
       <c r="M37" t="n">
-        <v>29599</v>
+        <v>34753</v>
       </c>
       <c r="N37" t="n">
-        <v>53804</v>
+        <v>60435</v>
       </c>
     </row>
     <row r="38">
@@ -2119,13 +2119,13 @@
         <v>7829</v>
       </c>
       <c r="L38" t="n">
-        <v>18338</v>
+        <v>20760</v>
       </c>
       <c r="M38" t="n">
-        <v>3149</v>
+        <v>3769</v>
       </c>
       <c r="N38" t="n">
-        <v>15189</v>
+        <v>16991</v>
       </c>
     </row>
     <row r="39">
@@ -2163,13 +2163,13 @@
         <v>26289</v>
       </c>
       <c r="L39" t="n">
-        <v>19747</v>
+        <v>22353</v>
       </c>
       <c r="M39" t="n">
-        <v>4294</v>
+        <v>4872</v>
       </c>
       <c r="N39" t="n">
-        <v>15453</v>
+        <v>17481</v>
       </c>
     </row>
     <row r="40">
@@ -2207,13 +2207,13 @@
         <v>74072</v>
       </c>
       <c r="L40" t="n">
-        <v>56732</v>
+        <v>64319</v>
       </c>
       <c r="M40" t="n">
-        <v>10482</v>
+        <v>12167</v>
       </c>
       <c r="N40" t="n">
-        <v>46250</v>
+        <v>52152</v>
       </c>
     </row>
     <row r="41">
@@ -2251,13 +2251,13 @@
         <v>11564</v>
       </c>
       <c r="L41" t="n">
-        <v>8335</v>
+        <v>9346</v>
       </c>
       <c r="M41" t="n">
-        <v>1275</v>
+        <v>1495</v>
       </c>
       <c r="N41" t="n">
-        <v>7060</v>
+        <v>7851</v>
       </c>
     </row>
     <row r="42">
@@ -2295,13 +2295,13 @@
         <v>41594</v>
       </c>
       <c r="L42" t="n">
-        <v>59151</v>
+        <v>67141</v>
       </c>
       <c r="M42" t="n">
-        <v>12148</v>
+        <v>14382</v>
       </c>
       <c r="N42" t="n">
-        <v>47003</v>
+        <v>52759</v>
       </c>
     </row>
     <row r="43">
@@ -2339,13 +2339,13 @@
         <v>39097</v>
       </c>
       <c r="L43" t="n">
-        <v>41035</v>
+        <v>46365</v>
       </c>
       <c r="M43" t="n">
-        <v>9938</v>
+        <v>11715</v>
       </c>
       <c r="N43" t="n">
-        <v>31097</v>
+        <v>34650</v>
       </c>
     </row>
     <row r="44">
@@ -2383,13 +2383,13 @@
         <v>90813</v>
       </c>
       <c r="L44" t="n">
-        <v>75972</v>
+        <v>85429</v>
       </c>
       <c r="M44" t="n">
-        <v>21474</v>
+        <v>24755</v>
       </c>
       <c r="N44" t="n">
-        <v>54498</v>
+        <v>60674</v>
       </c>
     </row>
     <row r="45">
@@ -2427,13 +2427,13 @@
         <v>74362</v>
       </c>
       <c r="L45" t="n">
-        <v>55239</v>
+        <v>63736</v>
       </c>
       <c r="M45" t="n">
-        <v>11765</v>
+        <v>13916</v>
       </c>
       <c r="N45" t="n">
-        <v>43474</v>
+        <v>49820</v>
       </c>
     </row>
     <row r="46">
@@ -2471,13 +2471,13 @@
         <v>66503</v>
       </c>
       <c r="L46" t="n">
-        <v>70781</v>
+        <v>79330</v>
       </c>
       <c r="M46" t="n">
-        <v>12157</v>
+        <v>14552</v>
       </c>
       <c r="N46" t="n">
-        <v>58624</v>
+        <v>64778</v>
       </c>
     </row>
     <row r="47">
@@ -2515,13 +2515,13 @@
         <v>286539</v>
       </c>
       <c r="L47" t="n">
-        <v>140410</v>
+        <v>164506</v>
       </c>
       <c r="M47" t="n">
-        <v>58595</v>
+        <v>68203</v>
       </c>
       <c r="N47" t="n">
-        <v>81815</v>
+        <v>96303</v>
       </c>
     </row>
     <row r="48">
@@ -2559,13 +2559,13 @@
         <v>262442</v>
       </c>
       <c r="L48" t="n">
-        <v>140729</v>
+        <v>166717</v>
       </c>
       <c r="M48" t="n">
-        <v>58059</v>
+        <v>69018</v>
       </c>
       <c r="N48" t="n">
-        <v>82670</v>
+        <v>97699</v>
       </c>
     </row>
     <row r="49">
@@ -2603,13 +2603,13 @@
         <v>73813</v>
       </c>
       <c r="L49" t="n">
-        <v>52505</v>
+        <v>60090</v>
       </c>
       <c r="M49" t="n">
-        <v>15890</v>
+        <v>18453</v>
       </c>
       <c r="N49" t="n">
-        <v>36615</v>
+        <v>41637</v>
       </c>
     </row>
     <row r="50">
@@ -2647,13 +2647,13 @@
         <v>14115</v>
       </c>
       <c r="L50" t="n">
-        <v>43502</v>
+        <v>47880</v>
       </c>
       <c r="M50" t="n">
-        <v>5745</v>
+        <v>6725</v>
       </c>
       <c r="N50" t="n">
-        <v>37757</v>
+        <v>41155</v>
       </c>
     </row>
     <row r="51">
@@ -2691,13 +2691,13 @@
         <v>14887</v>
       </c>
       <c r="L51" t="n">
-        <v>21744</v>
+        <v>24717</v>
       </c>
       <c r="M51" t="n">
-        <v>4996</v>
+        <v>5869</v>
       </c>
       <c r="N51" t="n">
-        <v>16748</v>
+        <v>18848</v>
       </c>
     </row>
     <row r="52">
@@ -2735,13 +2735,13 @@
         <v>52222</v>
       </c>
       <c r="L52" t="n">
-        <v>52384</v>
+        <v>59453</v>
       </c>
       <c r="M52" t="n">
-        <v>13576</v>
+        <v>15999</v>
       </c>
       <c r="N52" t="n">
-        <v>38808</v>
+        <v>43454</v>
       </c>
     </row>
     <row r="53">
@@ -2779,13 +2779,13 @@
         <v>29739</v>
       </c>
       <c r="L53" t="n">
-        <v>37819</v>
+        <v>42753</v>
       </c>
       <c r="M53" t="n">
-        <v>9752</v>
+        <v>11352</v>
       </c>
       <c r="N53" t="n">
-        <v>28067</v>
+        <v>31401</v>
       </c>
     </row>
     <row r="54">
@@ -2823,13 +2823,13 @@
         <v>33755</v>
       </c>
       <c r="L54" t="n">
-        <v>34891</v>
+        <v>40966</v>
       </c>
       <c r="M54" t="n">
-        <v>8727</v>
+        <v>10466</v>
       </c>
       <c r="N54" t="n">
-        <v>26164</v>
+        <v>30500</v>
       </c>
     </row>
     <row r="55">
@@ -2867,13 +2867,13 @@
         <v>15489</v>
       </c>
       <c r="L55" t="n">
-        <v>12978</v>
+        <v>15269</v>
       </c>
       <c r="M55" t="n">
-        <v>3418</v>
+        <v>4121</v>
       </c>
       <c r="N55" t="n">
-        <v>9560</v>
+        <v>11148</v>
       </c>
     </row>
     <row r="56">
@@ -2911,13 +2911,13 @@
         <v>90057</v>
       </c>
       <c r="L56" t="n">
-        <v>69044</v>
+        <v>79079</v>
       </c>
       <c r="M56" t="n">
-        <v>17163</v>
+        <v>20458</v>
       </c>
       <c r="N56" t="n">
-        <v>51881</v>
+        <v>58621</v>
       </c>
     </row>
     <row r="57">
@@ -2955,13 +2955,13 @@
         <v>22869</v>
       </c>
       <c r="L57" t="n">
-        <v>25340</v>
+        <v>28987</v>
       </c>
       <c r="M57" t="n">
-        <v>5688</v>
+        <v>6771</v>
       </c>
       <c r="N57" t="n">
-        <v>19652</v>
+        <v>22216</v>
       </c>
     </row>
     <row r="58">
@@ -2999,13 +2999,13 @@
         <v>50900</v>
       </c>
       <c r="L58" t="n">
-        <v>79658</v>
+        <v>90027</v>
       </c>
       <c r="M58" t="n">
-        <v>16252</v>
+        <v>19654</v>
       </c>
       <c r="N58" t="n">
-        <v>63406</v>
+        <v>70373</v>
       </c>
     </row>
     <row r="59">
@@ -3043,13 +3043,13 @@
         <v>57445</v>
       </c>
       <c r="L59" t="n">
-        <v>46292</v>
+        <v>53354</v>
       </c>
       <c r="M59" t="n">
-        <v>13229</v>
+        <v>15640</v>
       </c>
       <c r="N59" t="n">
-        <v>33063</v>
+        <v>37714</v>
       </c>
     </row>
     <row r="60">
@@ -3087,13 +3087,13 @@
         <v>64646</v>
       </c>
       <c r="L60" t="n">
-        <v>78332</v>
+        <v>91484</v>
       </c>
       <c r="M60" t="n">
-        <v>23220</v>
+        <v>28129</v>
       </c>
       <c r="N60" t="n">
-        <v>55112</v>
+        <v>63355</v>
       </c>
     </row>
     <row r="61">
@@ -3131,13 +3131,13 @@
         <v>29176</v>
       </c>
       <c r="L61" t="n">
-        <v>26506</v>
+        <v>30369</v>
       </c>
       <c r="M61" t="n">
-        <v>6683</v>
+        <v>7828</v>
       </c>
       <c r="N61" t="n">
-        <v>19823</v>
+        <v>22541</v>
       </c>
     </row>
     <row r="62">
@@ -3175,13 +3175,13 @@
         <v>25083</v>
       </c>
       <c r="L62" t="n">
-        <v>45221</v>
+        <v>51137</v>
       </c>
       <c r="M62" t="n">
-        <v>6672</v>
+        <v>8000</v>
       </c>
       <c r="N62" t="n">
-        <v>38549</v>
+        <v>43137</v>
       </c>
     </row>
     <row r="63">
@@ -3219,13 +3219,13 @@
         <v>20109</v>
       </c>
       <c r="L63" t="n">
-        <v>26589</v>
+        <v>30214</v>
       </c>
       <c r="M63" t="n">
-        <v>3864</v>
+        <v>4616</v>
       </c>
       <c r="N63" t="n">
-        <v>22725</v>
+        <v>25598</v>
       </c>
     </row>
     <row r="64">
@@ -3263,13 +3263,13 @@
         <v>35709</v>
       </c>
       <c r="L64" t="n">
-        <v>26935</v>
+        <v>30821</v>
       </c>
       <c r="M64" t="n">
-        <v>4922</v>
+        <v>5930</v>
       </c>
       <c r="N64" t="n">
-        <v>22013</v>
+        <v>24891</v>
       </c>
     </row>
     <row r="65">
@@ -3307,13 +3307,13 @@
         <v>69002</v>
       </c>
       <c r="L65" t="n">
-        <v>54447</v>
+        <v>62227</v>
       </c>
       <c r="M65" t="n">
-        <v>11380</v>
+        <v>13788</v>
       </c>
       <c r="N65" t="n">
-        <v>43067</v>
+        <v>48439</v>
       </c>
     </row>
     <row r="66">
@@ -3351,13 +3351,13 @@
         <v>85499</v>
       </c>
       <c r="L66" t="n">
-        <v>57565</v>
+        <v>66080</v>
       </c>
       <c r="M66" t="n">
-        <v>11579</v>
+        <v>13351</v>
       </c>
       <c r="N66" t="n">
-        <v>45986</v>
+        <v>52729</v>
       </c>
     </row>
     <row r="67">
@@ -3395,13 +3395,13 @@
         <v>27583</v>
       </c>
       <c r="L67" t="n">
-        <v>41532</v>
+        <v>48097</v>
       </c>
       <c r="M67" t="n">
-        <v>12760</v>
+        <v>15272</v>
       </c>
       <c r="N67" t="n">
-        <v>28772</v>
+        <v>32825</v>
       </c>
     </row>
     <row r="68">
@@ -3439,13 +3439,13 @@
         <v>42869</v>
       </c>
       <c r="L68" t="n">
-        <v>42400</v>
+        <v>49330</v>
       </c>
       <c r="M68" t="n">
-        <v>9064</v>
+        <v>10894</v>
       </c>
       <c r="N68" t="n">
-        <v>33336</v>
+        <v>38436</v>
       </c>
     </row>
     <row r="69">
@@ -3483,13 +3483,13 @@
         <v>78610</v>
       </c>
       <c r="L69" t="n">
-        <v>60845</v>
+        <v>70515</v>
       </c>
       <c r="M69" t="n">
-        <v>10127</v>
+        <v>12319</v>
       </c>
       <c r="N69" t="n">
-        <v>50718</v>
+        <v>58196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: data for 20260430, regenerated reports
</commit_message>
<xml_diff>
--- a/f_total_cap_nhat.xlsx
+++ b/f_total_cap_nhat.xlsx
@@ -535,13 +535,13 @@
         <v>150469</v>
       </c>
       <c r="L2" t="n">
-        <v>77543</v>
+        <v>85966</v>
       </c>
       <c r="M2" t="n">
-        <v>18149</v>
+        <v>21659</v>
       </c>
       <c r="N2" t="n">
-        <v>59394</v>
+        <v>64307</v>
       </c>
     </row>
     <row r="3">
@@ -579,13 +579,13 @@
         <v>81428</v>
       </c>
       <c r="L3" t="n">
-        <v>124018</v>
+        <v>140160</v>
       </c>
       <c r="M3" t="n">
-        <v>51469</v>
+        <v>60665</v>
       </c>
       <c r="N3" t="n">
-        <v>72549</v>
+        <v>79495</v>
       </c>
     </row>
     <row r="4">
@@ -623,13 +623,13 @@
         <v>18713</v>
       </c>
       <c r="L4" t="n">
-        <v>22541</v>
+        <v>24160</v>
       </c>
       <c r="M4" t="n">
-        <v>4275</v>
+        <v>4940</v>
       </c>
       <c r="N4" t="n">
-        <v>18266</v>
+        <v>19220</v>
       </c>
     </row>
     <row r="5">
@@ -667,13 +667,13 @@
         <v>42408</v>
       </c>
       <c r="L5" t="n">
-        <v>28201</v>
+        <v>30808</v>
       </c>
       <c r="M5" t="n">
-        <v>7661</v>
+        <v>8728</v>
       </c>
       <c r="N5" t="n">
-        <v>20540</v>
+        <v>22080</v>
       </c>
     </row>
     <row r="6">
@@ -711,13 +711,13 @@
         <v>117439</v>
       </c>
       <c r="L6" t="n">
-        <v>81432</v>
+        <v>89042</v>
       </c>
       <c r="M6" t="n">
-        <v>19477</v>
+        <v>22326</v>
       </c>
       <c r="N6" t="n">
-        <v>61955</v>
+        <v>66716</v>
       </c>
     </row>
     <row r="7">
@@ -755,13 +755,13 @@
         <v>19076</v>
       </c>
       <c r="L7" t="n">
-        <v>11156</v>
+        <v>12519</v>
       </c>
       <c r="M7" t="n">
-        <v>1914</v>
+        <v>2290</v>
       </c>
       <c r="N7" t="n">
-        <v>9242</v>
+        <v>10229</v>
       </c>
     </row>
     <row r="8">
@@ -799,13 +799,13 @@
         <v>83014</v>
       </c>
       <c r="L8" t="n">
-        <v>76229</v>
+        <v>83803</v>
       </c>
       <c r="M8" t="n">
-        <v>17609</v>
+        <v>20864</v>
       </c>
       <c r="N8" t="n">
-        <v>58620</v>
+        <v>62939</v>
       </c>
     </row>
     <row r="9">
@@ -843,13 +843,13 @@
         <v>65107</v>
       </c>
       <c r="L9" t="n">
-        <v>57115</v>
+        <v>62936</v>
       </c>
       <c r="M9" t="n">
-        <v>18127</v>
+        <v>20983</v>
       </c>
       <c r="N9" t="n">
-        <v>38988</v>
+        <v>41953</v>
       </c>
     </row>
     <row r="10">
@@ -887,13 +887,13 @@
         <v>151451</v>
       </c>
       <c r="L10" t="n">
-        <v>105517</v>
+        <v>115876</v>
       </c>
       <c r="M10" t="n">
-        <v>35942</v>
+        <v>41671</v>
       </c>
       <c r="N10" t="n">
-        <v>69575</v>
+        <v>74205</v>
       </c>
     </row>
     <row r="11">
@@ -931,13 +931,13 @@
         <v>127517</v>
       </c>
       <c r="L11" t="n">
-        <v>77837</v>
+        <v>86860</v>
       </c>
       <c r="M11" t="n">
-        <v>19426</v>
+        <v>23185</v>
       </c>
       <c r="N11" t="n">
-        <v>58411</v>
+        <v>63675</v>
       </c>
     </row>
     <row r="12">
@@ -975,13 +975,13 @@
         <v>122266</v>
       </c>
       <c r="L12" t="n">
-        <v>90980</v>
+        <v>100972</v>
       </c>
       <c r="M12" t="n">
-        <v>18585</v>
+        <v>22552</v>
       </c>
       <c r="N12" t="n">
-        <v>72395</v>
+        <v>78420</v>
       </c>
     </row>
     <row r="13">
@@ -1019,13 +1019,13 @@
         <v>399425</v>
       </c>
       <c r="L13" t="n">
-        <v>251605</v>
+        <v>278129</v>
       </c>
       <c r="M13" t="n">
-        <v>123936</v>
+        <v>140691</v>
       </c>
       <c r="N13" t="n">
-        <v>127669</v>
+        <v>137438</v>
       </c>
     </row>
     <row r="14">
@@ -1063,13 +1063,13 @@
         <v>274795</v>
       </c>
       <c r="L14" t="n">
-        <v>284549</v>
+        <v>320675</v>
       </c>
       <c r="M14" t="n">
-        <v>137420</v>
+        <v>159854</v>
       </c>
       <c r="N14" t="n">
-        <v>147129</v>
+        <v>160821</v>
       </c>
     </row>
     <row r="15">
@@ -1107,13 +1107,13 @@
         <v>80530</v>
       </c>
       <c r="L15" t="n">
-        <v>86966</v>
+        <v>99160</v>
       </c>
       <c r="M15" t="n">
-        <v>31265</v>
+        <v>37259</v>
       </c>
       <c r="N15" t="n">
-        <v>55701</v>
+        <v>61901</v>
       </c>
     </row>
     <row r="16">
@@ -1151,13 +1151,13 @@
         <v>15975</v>
       </c>
       <c r="L16" t="n">
-        <v>56679</v>
+        <v>63067</v>
       </c>
       <c r="M16" t="n">
-        <v>9262</v>
+        <v>10966</v>
       </c>
       <c r="N16" t="n">
-        <v>47417</v>
+        <v>52101</v>
       </c>
     </row>
     <row r="17">
@@ -1195,13 +1195,13 @@
         <v>26564</v>
       </c>
       <c r="L17" t="n">
-        <v>30510</v>
+        <v>33399</v>
       </c>
       <c r="M17" t="n">
-        <v>8858</v>
+        <v>10302</v>
       </c>
       <c r="N17" t="n">
-        <v>21652</v>
+        <v>23097</v>
       </c>
     </row>
     <row r="18">
@@ -1239,13 +1239,13 @@
         <v>66764</v>
       </c>
       <c r="L18" t="n">
-        <v>81004</v>
+        <v>92263</v>
       </c>
       <c r="M18" t="n">
-        <v>25646</v>
+        <v>30719</v>
       </c>
       <c r="N18" t="n">
-        <v>55358</v>
+        <v>61544</v>
       </c>
     </row>
     <row r="19">
@@ -1283,13 +1283,13 @@
         <v>55231</v>
       </c>
       <c r="L19" t="n">
-        <v>49519</v>
+        <v>54396</v>
       </c>
       <c r="M19" t="n">
-        <v>14742</v>
+        <v>17126</v>
       </c>
       <c r="N19" t="n">
-        <v>34777</v>
+        <v>37270</v>
       </c>
     </row>
     <row r="20">
@@ -1327,13 +1327,13 @@
         <v>58737</v>
       </c>
       <c r="L20" t="n">
-        <v>47231</v>
+        <v>53877</v>
       </c>
       <c r="M20" t="n">
-        <v>12557</v>
+        <v>15291</v>
       </c>
       <c r="N20" t="n">
-        <v>34674</v>
+        <v>38586</v>
       </c>
     </row>
     <row r="21">
@@ -1371,13 +1371,13 @@
         <v>24382</v>
       </c>
       <c r="L21" t="n">
-        <v>18358</v>
+        <v>20689</v>
       </c>
       <c r="M21" t="n">
-        <v>5128</v>
+        <v>5894</v>
       </c>
       <c r="N21" t="n">
-        <v>13230</v>
+        <v>14795</v>
       </c>
     </row>
     <row r="22">
@@ -1415,13 +1415,13 @@
         <v>152229</v>
       </c>
       <c r="L22" t="n">
-        <v>91008</v>
+        <v>101195</v>
       </c>
       <c r="M22" t="n">
-        <v>25839</v>
+        <v>31048</v>
       </c>
       <c r="N22" t="n">
-        <v>65169</v>
+        <v>70147</v>
       </c>
     </row>
     <row r="23">
@@ -1459,13 +1459,13 @@
         <v>40867</v>
       </c>
       <c r="L23" t="n">
-        <v>33044</v>
+        <v>37369</v>
       </c>
       <c r="M23" t="n">
-        <v>8117</v>
+        <v>9886</v>
       </c>
       <c r="N23" t="n">
-        <v>24927</v>
+        <v>27483</v>
       </c>
     </row>
     <row r="24">
@@ -1503,13 +1503,13 @@
         <v>88798</v>
       </c>
       <c r="L24" t="n">
-        <v>106760</v>
+        <v>121362</v>
       </c>
       <c r="M24" t="n">
-        <v>26787</v>
+        <v>32879</v>
       </c>
       <c r="N24" t="n">
-        <v>79973</v>
+        <v>88483</v>
       </c>
     </row>
     <row r="25">
@@ -1547,13 +1547,13 @@
         <v>86600</v>
       </c>
       <c r="L25" t="n">
-        <v>74479</v>
+        <v>85819</v>
       </c>
       <c r="M25" t="n">
-        <v>26124</v>
+        <v>31958</v>
       </c>
       <c r="N25" t="n">
-        <v>48355</v>
+        <v>53861</v>
       </c>
     </row>
     <row r="26">
@@ -1591,13 +1591,13 @@
         <v>95605</v>
       </c>
       <c r="L26" t="n">
-        <v>114529</v>
+        <v>134161</v>
       </c>
       <c r="M26" t="n">
-        <v>39114</v>
+        <v>48677</v>
       </c>
       <c r="N26" t="n">
-        <v>75415</v>
+        <v>85484</v>
       </c>
     </row>
     <row r="27">
@@ -1635,13 +1635,13 @@
         <v>35197</v>
       </c>
       <c r="L27" t="n">
-        <v>40234</v>
+        <v>44329</v>
       </c>
       <c r="M27" t="n">
-        <v>11858</v>
+        <v>13756</v>
       </c>
       <c r="N27" t="n">
-        <v>28376</v>
+        <v>30573</v>
       </c>
     </row>
     <row r="28">
@@ -1679,13 +1679,13 @@
         <v>52800</v>
       </c>
       <c r="L28" t="n">
-        <v>56855</v>
+        <v>62106</v>
       </c>
       <c r="M28" t="n">
-        <v>10163</v>
+        <v>12058</v>
       </c>
       <c r="N28" t="n">
-        <v>46692</v>
+        <v>50048</v>
       </c>
     </row>
     <row r="29">
@@ -1723,13 +1723,13 @@
         <v>34093</v>
       </c>
       <c r="L29" t="n">
-        <v>36559</v>
+        <v>40551</v>
       </c>
       <c r="M29" t="n">
-        <v>6482</v>
+        <v>7705</v>
       </c>
       <c r="N29" t="n">
-        <v>30077</v>
+        <v>32846</v>
       </c>
     </row>
     <row r="30">
@@ -1767,13 +1767,13 @@
         <v>59519</v>
       </c>
       <c r="L30" t="n">
-        <v>35366</v>
+        <v>40087</v>
       </c>
       <c r="M30" t="n">
-        <v>7164</v>
+        <v>9103</v>
       </c>
       <c r="N30" t="n">
-        <v>28202</v>
+        <v>30984</v>
       </c>
     </row>
     <row r="31">
@@ -1811,13 +1811,13 @@
         <v>111215</v>
       </c>
       <c r="L31" t="n">
-        <v>77984</v>
+        <v>88709</v>
       </c>
       <c r="M31" t="n">
-        <v>19970</v>
+        <v>24678</v>
       </c>
       <c r="N31" t="n">
-        <v>58014</v>
+        <v>64031</v>
       </c>
     </row>
     <row r="32">
@@ -1855,13 +1855,13 @@
         <v>135620</v>
       </c>
       <c r="L32" t="n">
-        <v>84651</v>
+        <v>93200</v>
       </c>
       <c r="M32" t="n">
-        <v>20965</v>
+        <v>24512</v>
       </c>
       <c r="N32" t="n">
-        <v>63686</v>
+        <v>68688</v>
       </c>
     </row>
     <row r="33">
@@ -1899,13 +1899,13 @@
         <v>46108</v>
       </c>
       <c r="L33" t="n">
-        <v>56833</v>
+        <v>64341</v>
       </c>
       <c r="M33" t="n">
-        <v>19978</v>
+        <v>24063</v>
       </c>
       <c r="N33" t="n">
-        <v>36855</v>
+        <v>40278</v>
       </c>
     </row>
     <row r="34">
@@ -1943,13 +1943,13 @@
         <v>74035</v>
       </c>
       <c r="L34" t="n">
-        <v>56342</v>
+        <v>64598</v>
       </c>
       <c r="M34" t="n">
-        <v>12814</v>
+        <v>15594</v>
       </c>
       <c r="N34" t="n">
-        <v>43528</v>
+        <v>49004</v>
       </c>
     </row>
     <row r="35">
@@ -1987,13 +1987,13 @@
         <v>134411</v>
       </c>
       <c r="L35" t="n">
-        <v>84616</v>
+        <v>94162</v>
       </c>
       <c r="M35" t="n">
-        <v>17861</v>
+        <v>21343</v>
       </c>
       <c r="N35" t="n">
-        <v>66755</v>
+        <v>72819</v>
       </c>
     </row>
     <row r="36">
@@ -2031,13 +2031,13 @@
         <v>93875</v>
       </c>
       <c r="L36" t="n">
-        <v>61912</v>
+        <v>68260</v>
       </c>
       <c r="M36" t="n">
-        <v>12594</v>
+        <v>15050</v>
       </c>
       <c r="N36" t="n">
-        <v>49318</v>
+        <v>53210</v>
       </c>
     </row>
     <row r="37">
@@ -2075,13 +2075,13 @@
         <v>65690</v>
       </c>
       <c r="L37" t="n">
-        <v>95188</v>
+        <v>107273</v>
       </c>
       <c r="M37" t="n">
-        <v>34753</v>
+        <v>41243</v>
       </c>
       <c r="N37" t="n">
-        <v>60435</v>
+        <v>66030</v>
       </c>
     </row>
     <row r="38">
@@ -2119,13 +2119,13 @@
         <v>7829</v>
       </c>
       <c r="L38" t="n">
-        <v>20760</v>
+        <v>22203</v>
       </c>
       <c r="M38" t="n">
-        <v>3769</v>
+        <v>4353</v>
       </c>
       <c r="N38" t="n">
-        <v>16991</v>
+        <v>17850</v>
       </c>
     </row>
     <row r="39">
@@ -2163,13 +2163,13 @@
         <v>26289</v>
       </c>
       <c r="L39" t="n">
-        <v>22353</v>
+        <v>24301</v>
       </c>
       <c r="M39" t="n">
-        <v>4872</v>
+        <v>5557</v>
       </c>
       <c r="N39" t="n">
-        <v>17481</v>
+        <v>18744</v>
       </c>
     </row>
     <row r="40">
@@ -2207,13 +2207,13 @@
         <v>74072</v>
       </c>
       <c r="L40" t="n">
-        <v>64319</v>
+        <v>69865</v>
       </c>
       <c r="M40" t="n">
-        <v>12167</v>
+        <v>13942</v>
       </c>
       <c r="N40" t="n">
-        <v>52152</v>
+        <v>55923</v>
       </c>
     </row>
     <row r="41">
@@ -2251,13 +2251,13 @@
         <v>11564</v>
       </c>
       <c r="L41" t="n">
-        <v>9346</v>
+        <v>10453</v>
       </c>
       <c r="M41" t="n">
-        <v>1495</v>
+        <v>1804</v>
       </c>
       <c r="N41" t="n">
-        <v>7851</v>
+        <v>8649</v>
       </c>
     </row>
     <row r="42">
@@ -2295,13 +2295,13 @@
         <v>41594</v>
       </c>
       <c r="L42" t="n">
-        <v>67141</v>
+        <v>73521</v>
       </c>
       <c r="M42" t="n">
-        <v>14382</v>
+        <v>17064</v>
       </c>
       <c r="N42" t="n">
-        <v>52759</v>
+        <v>56457</v>
       </c>
     </row>
     <row r="43">
@@ -2339,13 +2339,13 @@
         <v>39097</v>
       </c>
       <c r="L43" t="n">
-        <v>46365</v>
+        <v>50819</v>
       </c>
       <c r="M43" t="n">
-        <v>11715</v>
+        <v>13659</v>
       </c>
       <c r="N43" t="n">
-        <v>34650</v>
+        <v>37160</v>
       </c>
     </row>
     <row r="44">
@@ -2383,13 +2383,13 @@
         <v>90813</v>
       </c>
       <c r="L44" t="n">
-        <v>85429</v>
+        <v>93302</v>
       </c>
       <c r="M44" t="n">
-        <v>24755</v>
+        <v>28804</v>
       </c>
       <c r="N44" t="n">
-        <v>60674</v>
+        <v>64498</v>
       </c>
     </row>
     <row r="45">
@@ -2427,13 +2427,13 @@
         <v>74362</v>
       </c>
       <c r="L45" t="n">
-        <v>63736</v>
+        <v>70818</v>
       </c>
       <c r="M45" t="n">
-        <v>13916</v>
+        <v>16680</v>
       </c>
       <c r="N45" t="n">
-        <v>49820</v>
+        <v>54138</v>
       </c>
     </row>
     <row r="46">
@@ -2471,13 +2471,13 @@
         <v>66503</v>
       </c>
       <c r="L46" t="n">
-        <v>79330</v>
+        <v>87642</v>
       </c>
       <c r="M46" t="n">
-        <v>14552</v>
+        <v>17682</v>
       </c>
       <c r="N46" t="n">
-        <v>64778</v>
+        <v>69960</v>
       </c>
     </row>
     <row r="47">
@@ -2515,13 +2515,13 @@
         <v>286539</v>
       </c>
       <c r="L47" t="n">
-        <v>164506</v>
+        <v>181434</v>
       </c>
       <c r="M47" t="n">
-        <v>68203</v>
+        <v>77966</v>
       </c>
       <c r="N47" t="n">
-        <v>96303</v>
+        <v>103468</v>
       </c>
     </row>
     <row r="48">
@@ -2559,13 +2559,13 @@
         <v>262442</v>
       </c>
       <c r="L48" t="n">
-        <v>166717</v>
+        <v>187520</v>
       </c>
       <c r="M48" t="n">
-        <v>69018</v>
+        <v>80961</v>
       </c>
       <c r="N48" t="n">
-        <v>97699</v>
+        <v>106559</v>
       </c>
     </row>
     <row r="49">
@@ -2603,13 +2603,13 @@
         <v>73813</v>
       </c>
       <c r="L49" t="n">
-        <v>60090</v>
+        <v>67923</v>
       </c>
       <c r="M49" t="n">
-        <v>18453</v>
+        <v>21973</v>
       </c>
       <c r="N49" t="n">
-        <v>41637</v>
+        <v>45950</v>
       </c>
     </row>
     <row r="50">
@@ -2647,13 +2647,13 @@
         <v>14115</v>
       </c>
       <c r="L50" t="n">
-        <v>47880</v>
+        <v>53082</v>
       </c>
       <c r="M50" t="n">
-        <v>6725</v>
+        <v>7998</v>
       </c>
       <c r="N50" t="n">
-        <v>41155</v>
+        <v>45084</v>
       </c>
     </row>
     <row r="51">
@@ -2691,13 +2691,13 @@
         <v>14887</v>
       </c>
       <c r="L51" t="n">
-        <v>24717</v>
+        <v>26848</v>
       </c>
       <c r="M51" t="n">
-        <v>5869</v>
+        <v>6817</v>
       </c>
       <c r="N51" t="n">
-        <v>18848</v>
+        <v>20031</v>
       </c>
     </row>
     <row r="52">
@@ -2735,13 +2735,13 @@
         <v>52222</v>
       </c>
       <c r="L52" t="n">
-        <v>59453</v>
+        <v>67178</v>
       </c>
       <c r="M52" t="n">
-        <v>15999</v>
+        <v>19284</v>
       </c>
       <c r="N52" t="n">
-        <v>43454</v>
+        <v>47894</v>
       </c>
     </row>
     <row r="53">
@@ -2779,13 +2779,13 @@
         <v>29739</v>
       </c>
       <c r="L53" t="n">
-        <v>42753</v>
+        <v>46715</v>
       </c>
       <c r="M53" t="n">
-        <v>11352</v>
+        <v>13156</v>
       </c>
       <c r="N53" t="n">
-        <v>31401</v>
+        <v>33559</v>
       </c>
     </row>
     <row r="54">
@@ -2823,13 +2823,13 @@
         <v>33755</v>
       </c>
       <c r="L54" t="n">
-        <v>40966</v>
+        <v>46525</v>
       </c>
       <c r="M54" t="n">
-        <v>10466</v>
+        <v>12763</v>
       </c>
       <c r="N54" t="n">
-        <v>30500</v>
+        <v>33762</v>
       </c>
     </row>
     <row r="55">
@@ -2867,13 +2867,13 @@
         <v>15489</v>
       </c>
       <c r="L55" t="n">
-        <v>15269</v>
+        <v>17206</v>
       </c>
       <c r="M55" t="n">
-        <v>4121</v>
+        <v>4753</v>
       </c>
       <c r="N55" t="n">
-        <v>11148</v>
+        <v>12453</v>
       </c>
     </row>
     <row r="56">
@@ -2911,13 +2911,13 @@
         <v>90057</v>
       </c>
       <c r="L56" t="n">
-        <v>79079</v>
+        <v>87572</v>
       </c>
       <c r="M56" t="n">
-        <v>20458</v>
+        <v>24692</v>
       </c>
       <c r="N56" t="n">
-        <v>58621</v>
+        <v>62880</v>
       </c>
     </row>
     <row r="57">
@@ -2955,13 +2955,13 @@
         <v>22869</v>
       </c>
       <c r="L57" t="n">
-        <v>28987</v>
+        <v>32674</v>
       </c>
       <c r="M57" t="n">
-        <v>6771</v>
+        <v>8272</v>
       </c>
       <c r="N57" t="n">
-        <v>22216</v>
+        <v>24402</v>
       </c>
     </row>
     <row r="58">
@@ -2999,13 +2999,13 @@
         <v>50900</v>
       </c>
       <c r="L58" t="n">
-        <v>90027</v>
+        <v>101727</v>
       </c>
       <c r="M58" t="n">
-        <v>19654</v>
+        <v>24233</v>
       </c>
       <c r="N58" t="n">
-        <v>70373</v>
+        <v>77494</v>
       </c>
     </row>
     <row r="59">
@@ -3043,13 +3043,13 @@
         <v>57445</v>
       </c>
       <c r="L59" t="n">
-        <v>53354</v>
+        <v>61157</v>
       </c>
       <c r="M59" t="n">
-        <v>15640</v>
+        <v>19373</v>
       </c>
       <c r="N59" t="n">
-        <v>37714</v>
+        <v>41784</v>
       </c>
     </row>
     <row r="60">
@@ -3087,13 +3087,13 @@
         <v>64646</v>
       </c>
       <c r="L60" t="n">
-        <v>91484</v>
+        <v>106780</v>
       </c>
       <c r="M60" t="n">
-        <v>28129</v>
+        <v>35314</v>
       </c>
       <c r="N60" t="n">
-        <v>63355</v>
+        <v>71466</v>
       </c>
     </row>
     <row r="61">
@@ -3131,13 +3131,13 @@
         <v>29176</v>
       </c>
       <c r="L61" t="n">
-        <v>30369</v>
+        <v>33279</v>
       </c>
       <c r="M61" t="n">
-        <v>7828</v>
+        <v>9063</v>
       </c>
       <c r="N61" t="n">
-        <v>22541</v>
+        <v>24216</v>
       </c>
     </row>
     <row r="62">
@@ -3175,13 +3175,13 @@
         <v>25083</v>
       </c>
       <c r="L62" t="n">
-        <v>51137</v>
+        <v>55573</v>
       </c>
       <c r="M62" t="n">
-        <v>8000</v>
+        <v>9502</v>
       </c>
       <c r="N62" t="n">
-        <v>43137</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="63">
@@ -3219,13 +3219,13 @@
         <v>20109</v>
       </c>
       <c r="L63" t="n">
-        <v>30214</v>
+        <v>33317</v>
       </c>
       <c r="M63" t="n">
-        <v>4616</v>
+        <v>5481</v>
       </c>
       <c r="N63" t="n">
-        <v>25598</v>
+        <v>27836</v>
       </c>
     </row>
     <row r="64">
@@ -3263,13 +3263,13 @@
         <v>35709</v>
       </c>
       <c r="L64" t="n">
-        <v>30821</v>
+        <v>34705</v>
       </c>
       <c r="M64" t="n">
-        <v>5930</v>
+        <v>7516</v>
       </c>
       <c r="N64" t="n">
-        <v>24891</v>
+        <v>27189</v>
       </c>
     </row>
     <row r="65">
@@ -3307,13 +3307,13 @@
         <v>69002</v>
       </c>
       <c r="L65" t="n">
-        <v>62227</v>
+        <v>70364</v>
       </c>
       <c r="M65" t="n">
-        <v>13788</v>
+        <v>17183</v>
       </c>
       <c r="N65" t="n">
-        <v>48439</v>
+        <v>53181</v>
       </c>
     </row>
     <row r="66">
@@ -3351,13 +3351,13 @@
         <v>85499</v>
       </c>
       <c r="L66" t="n">
-        <v>66080</v>
+        <v>72339</v>
       </c>
       <c r="M66" t="n">
-        <v>13351</v>
+        <v>15696</v>
       </c>
       <c r="N66" t="n">
-        <v>52729</v>
+        <v>56643</v>
       </c>
     </row>
     <row r="67">
@@ -3395,13 +3395,13 @@
         <v>27583</v>
       </c>
       <c r="L67" t="n">
-        <v>48097</v>
+        <v>54239</v>
       </c>
       <c r="M67" t="n">
-        <v>15272</v>
+        <v>18491</v>
       </c>
       <c r="N67" t="n">
-        <v>32825</v>
+        <v>35748</v>
       </c>
     </row>
     <row r="68">
@@ -3439,13 +3439,13 @@
         <v>42869</v>
       </c>
       <c r="L68" t="n">
-        <v>49330</v>
+        <v>56222</v>
       </c>
       <c r="M68" t="n">
-        <v>10894</v>
+        <v>13244</v>
       </c>
       <c r="N68" t="n">
-        <v>38436</v>
+        <v>42978</v>
       </c>
     </row>
     <row r="69">
@@ -3483,13 +3483,13 @@
         <v>78610</v>
       </c>
       <c r="L69" t="n">
-        <v>70515</v>
+        <v>78079</v>
       </c>
       <c r="M69" t="n">
-        <v>12319</v>
+        <v>14803</v>
       </c>
       <c r="N69" t="n">
-        <v>58196</v>
+        <v>63276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>